<commit_message>
updated for log message
</commit_message>
<xml_diff>
--- a/data/target/customer_100003_002.xlsx
+++ b/data/target/customer_100003_002.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Downloads\easyexcelcomparator\data\target\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF0BC781-9033-438D-B551-CCA36D5AC1DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F4AF138-EDA6-4CDD-974C-8C6CB42DBCC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{49010DB3-58E0-4DBF-ADA8-C1E2291ECC60}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="9">
   <si>
     <t xml:space="preserve">Name </t>
   </si>
@@ -422,7 +422,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6605A4E-8B79-4106-92C3-0B944BF1B2AB}">
-  <dimension ref="A2:E5"/>
+  <dimension ref="A2:E6"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="6.33203125" bestFit="1" customWidth="1"/>
@@ -455,12 +455,12 @@
         <v>30</v>
       </c>
       <c r="C3" s="2">
-        <f t="shared" ref="C3:D5" ca="1" si="0">NOW()</f>
-        <v>46294.983770254628</v>
+        <f t="shared" ref="C3:D6" ca="1" si="0">NOW()</f>
+        <v>46295.830446064814</v>
       </c>
       <c r="D3" s="2">
         <f t="shared" ca="1" si="0"/>
-        <v>46294.983770254628</v>
+        <v>46295.830446064814</v>
       </c>
       <c r="E3">
         <v>4</v>
@@ -475,11 +475,11 @@
       </c>
       <c r="C4" s="2">
         <f t="shared" ca="1" si="0"/>
-        <v>46294.983770254628</v>
+        <v>46295.830446064814</v>
       </c>
       <c r="D4" s="2">
         <f t="shared" ca="1" si="0"/>
-        <v>46294.983770254628</v>
+        <v>46295.830446064814</v>
       </c>
       <c r="E4">
         <v>5</v>
@@ -490,17 +490,35 @@
         <v>6</v>
       </c>
       <c r="B5">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C5" s="2">
         <f t="shared" ca="1" si="0"/>
-        <v>46294.983770254628</v>
+        <v>46295.830446064814</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E5">
         <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6">
+        <v>30</v>
+      </c>
+      <c r="C6" s="2">
+        <f t="shared" ca="1" si="0"/>
+        <v>46295.830446064814</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E6">
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>